<commit_message>
Add COMET full-sequence subtypes to distance exports
</commit_message>
<xml_diff>
--- a/HCVData/subtyping-comparison-all-ras/11-report-subtype-agreement/NS3_CometFullSeqSubtype_1L_Subtyping_Distances.xlsx
+++ b/HCVData/subtyping-comparison-all-ras/11-report-subtype-agreement/NS3_CometFullSeqSubtype_1L_Subtyping_Distances.xlsx
@@ -431,65 +431,70 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>CometFullSeqSubtype</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>ClosestSubtypeAlignedNT</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Genotype1Distance</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Genotype2Distance</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Genotype3Distance</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Genotype4Distance</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Genotype5Distance</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Genotype6Distance</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Genotype7Distance</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Genotype8Distance</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>FirstChoiceGenotype</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>FirstChoiceDistance</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>SecondChoiceGenotype</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>SecondChoiceDistance</t>
         </is>
@@ -503,65 +508,70 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>1L</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>2057</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>21.181</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>29.956</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>30.076</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>27.268</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>27.824</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>29.815</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>31.199</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>30.044</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>21.181</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>27.268</t>
         </is>
@@ -588,150 +598,155 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>CometFullSeqSubtype</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>ClosestSubtypeAlignedNT</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>AssignedGenotype</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Subtype1aDistance</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Subtype1aDistance</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Subtype1bDistance</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Subtype1bDistance</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Subtype1cDistance</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Subtype1cDistance</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Subtype1dDistance</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Subtype1eDistance</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Subtype1eDistance</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Subtype1gDistance</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Subtype1gDistance</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Subtype1hDistance</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Subtype1hDistance</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Subtype1iDistance</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Subtype1jDistance</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Subtype1kDistance</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Subtype1lDistance</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Subtype1lDistance</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Subtype1mDistance</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Subtype1mDistance</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Subtype1nDistance</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Subtype1nDistance</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>Subtype1oDistance</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>Subtype1oDistance</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>FirstChoiceSubtype</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>FirstChoiceDistance</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>SecondChoiceSubtype</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>SecondChoiceDistance</t>
         </is>
@@ -745,150 +760,155 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>1L</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>2057</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>20.986</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>20.986</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>20.603</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>20.603</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>22.255</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>22.255</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>22.368</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>23.073</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>23.073</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>22.754</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>22.754</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>21.415</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>21.415</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>22.233</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>22.499</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>22.071</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>16.869</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>16.869</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>21.665</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="X2" t="inlineStr">
         <is>
           <t>21.665</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
         <is>
           <t>22.049</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="Z2" t="inlineStr">
         <is>
           <t>22.049</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="AA2" t="inlineStr">
         <is>
           <t>21.230</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AB2" t="inlineStr">
         <is>
           <t>21.230</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>1l</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
         <is>
           <t>16.869</t>
         </is>
       </c>
-      <c r="AD2" t="inlineStr">
+      <c r="AE2" t="inlineStr">
         <is>
           <t>1b</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr">
+      <c r="AF2" t="inlineStr">
         <is>
           <t>20.603</t>
         </is>
@@ -915,145 +935,150 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>CometFullSeqSubtype</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>ClosestSubtypeAlignedNT</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>AssignedGenotype</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Subtype2aDistance</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Subtype2aDistance</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Subtype2bDistance</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Subtype2bDistance</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Subtype2cDistance</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Subtype2dDistance</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Subtype2eDistance</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Subtype2fDistance</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Subtype2fDistance</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Subtype2iDistance</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Subtype2jDistance</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Subtype2jDistance</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Subtype2kDistance</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Subtype2lDistance</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Subtype2lDistance</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Subtype2mDistance</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Subtype2mDistance</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Subtype2qDistance</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Subtype2qDistance</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Subtype2rDistance</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Subtype2tDistance</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Subtype2uDistance</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>Subtype2vDistance</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>FirstChoiceSubtype</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>FirstChoiceDistance</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>SecondChoiceSubtype</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>SecondChoiceDistance</t>
         </is>
@@ -1080,85 +1105,90 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>CometFullSeqSubtype</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>ClosestSubtypeAlignedNT</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>AssignedGenotype</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Subtype3aDistance</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Subtype3bDistance</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Subtype3dDistance</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Subtype3eDistance</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Subtype3gDistance</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Subtype3gDistance</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Subtype3hDistance</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Subtype3iDistance</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Subtype3iDistance</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Subtype3kDistance</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Subtype3kDistance</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>FirstChoiceSubtype</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>FirstChoiceDistance</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>SecondChoiceSubtype</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>SecondChoiceDistance</t>
         </is>
@@ -1185,145 +1215,150 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>CometFullSeqSubtype</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>ClosestSubtypeAlignedNT</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>AssignedGenotype</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Subtype4aDistance</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Subtype4bDistance</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Subtype4cDistance</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Subtype4dDistance</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Subtype4dDistance</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Subtype4fDistance</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Subtype4fDistance</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Subtype4gDistance</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Subtype4kDistance</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Subtype4kDistance</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Subtype4lDistance</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Subtype4mDistance</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Subtype4nDistance</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Subtype4oDistance</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Subtype4pDistance</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Subtype4qDistance</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Subtype4rDistance</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Subtype4sDistance</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Subtype4tDistance</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Subtype4vDistance</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Subtype4vDistance</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Subtype4wDistance</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>Subtype4wDistance</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>FirstChoiceSubtype</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>FirstChoiceDistance</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>SecondChoiceSubtype</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>SecondChoiceDistance</t>
         </is>
@@ -1350,40 +1385,45 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>CometFullSeqSubtype</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>ClosestSubtypeAlignedNT</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>AssignedGenotype</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Subtype5aDistance</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Subtype5bDistance</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>FirstChoiceSubtype</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>FirstChoiceDistance</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>SecondChoiceSubtype</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>SecondChoiceDistance</t>
         </is>
@@ -1410,255 +1450,260 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>CometFullSeqSubtype</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>ClosestSubtypeAlignedNT</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>AssignedGenotype</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Subtype6aDistance</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Subtype6aDistance</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Subtype6bDistance</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Subtype6cDistance</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Subtype6dDistance</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Subtype6eDistance</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Subtype6fDistance</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Subtype6gDistance</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Subtype6hDistance</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Subtype6iDistance</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Subtype6jDistance</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Subtype6kDistance</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Subtype6lDistance</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Subtype6mDistance</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Subtype6nDistance</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Subtype6nDistance</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Subtype6oDistance</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Subtype6pDistance</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Subtype6qDistance</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Subtype6rDistance</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Subtype6sDistance</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Subtype6tDistance</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>Subtype6tDistance</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>Subtype6uDistance</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>Subtype6vDistance</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>Subtype6vDistance</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>Subtype6wDistance</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>Subtype6wDistance</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>Subtype6xaDistance</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>Subtype6xaDistance</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>Subtype6xbDistance</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>Subtype6xbDistance</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>Subtype6xcDistance</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>Subtype6xdDistance</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>Subtype6xdDistance</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>Subtype6xeDistance</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>Subtype6xeDistance</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>Subtype6xfDistance</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>Subtype6xfDistance</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>Subtype6xgDistance</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>Subtype6xgDistance</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>Subtype6xhDistance</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>Subtype6xiDistance</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>Subtype6xiDistance</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>Subtype6xjDistance</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>FirstChoiceSubtype</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>FirstChoiceDistance</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>SecondChoiceSubtype</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>SecondChoiceDistance</t>
         </is>
@@ -1685,40 +1730,45 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>CometFullSeqSubtype</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>ClosestSubtypeAlignedNT</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>AssignedGenotype</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Subtype7aDistance</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Subtype7bDistance</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>FirstChoiceSubtype</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>FirstChoiceDistance</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>SecondChoiceSubtype</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>SecondChoiceDistance</t>
         </is>
@@ -1745,35 +1795,40 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>CometFullSeqSubtype</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>ClosestSubtypeAlignedNT</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>AssignedGenotype</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Subtype8aDistance</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>FirstChoiceSubtype</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>FirstChoiceDistance</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>SecondChoiceSubtype</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>SecondChoiceDistance</t>
         </is>

</xml_diff>